<commit_message>
add new product class script
</commit_message>
<xml_diff>
--- a/TestData/FloorFactory.xlsx
+++ b/TestData/FloorFactory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sashw\AutomationProjects\New folder\FloorFactoryP\FloorFactory\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B42B57-A42A-4D58-8313-64D4B7650A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8394281-2267-4475-83B6-9C92F8FC56DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{DDE78683-B506-475D-8992-C0E50F7FDFE3}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="58">
   <si>
     <t>Login Module</t>
   </si>
@@ -141,9 +141,6 @@
     <t>EmptyField</t>
   </si>
   <si>
-    <t>InterialFloaring</t>
-  </si>
-  <si>
     <t>C:\Users\sashw\AutomationProjects\New folder\FloorFactoryP\FloorFactory\src\test\resources\Images\CategoryImg.jpg</t>
   </si>
   <si>
@@ -153,7 +150,55 @@
     <t/>
   </si>
   <si>
-    <t>Interiar</t>
+    <t>Verify Edit Functionality</t>
+  </si>
+  <si>
+    <t>Delete Dunctionality</t>
+  </si>
+  <si>
+    <t>IsDeletedCategory</t>
+  </si>
+  <si>
+    <t>Factory</t>
+  </si>
+  <si>
+    <t>Factorysssss</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>box</t>
+  </si>
+  <si>
+    <t>"C:\Users\sashw\AutomationProjects\New folder\FloorFactoryP\FloorFactory\src\test\resources\Images\Subcategory.jpg"</t>
+  </si>
+  <si>
+    <t>Create new Subcategory with valid input</t>
+  </si>
+  <si>
+    <t>MCAA11</t>
+  </si>
+  <si>
+    <t>NDAA</t>
+  </si>
+  <si>
+    <t>SUBB</t>
+  </si>
+  <si>
+    <t>InActive</t>
+  </si>
+  <si>
+    <t>'"C:\Users\sashw\AutomationProjects\New folder\FloorFactoryP\FloorFactory\src\test\resources\Images\Subcategory.jpg"</t>
+  </si>
+  <si>
+    <t>Update SubCategory deatils</t>
+  </si>
+  <si>
+    <t>PVCCSub</t>
+  </si>
+  <si>
+    <t>C:\Users\sashw\AutomationProjects\New folder\FloorFactoryP\FloorFactory\src\test\resources\Images\Subcategory.jpg</t>
   </si>
 </sst>
 </file>
@@ -251,7 +296,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -274,6 +319,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -590,14 +638,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{545CD2D5-C1F8-4C88-8A29-C6004990FDF0}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.21875" customWidth="1"/>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
     <col min="3" max="3" width="30.5546875" customWidth="1"/>
     <col min="4" max="4" width="13.88671875" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -684,10 +732,10 @@
         <v>18</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="14" t="s">
         <v>38</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>39</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
@@ -699,7 +747,7 @@
         <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -707,14 +755,11 @@
       <c r="C9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D9" t="s">
-        <v>42</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -734,11 +779,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" s="7"/>
-      <c r="C11" s="9"/>
+      <c r="C11" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
-        <v>17</v>
+      <c r="B12" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -754,21 +813,23 @@
       <c r="C14" t="s">
         <v>24</v>
       </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C15" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="13" t="s">
+      <c r="D15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="B18" s="13"/>
       <c r="C18" s="13" t="s">
         <v>21</v>
       </c>
@@ -782,85 +843,125 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B19" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C20" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="C21" t="s">
+      <c r="C19" s="11"/>
+      <c r="D19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C20" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" t="s">
+        <v>54</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="D22" s="12"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="12"/>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="7" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D24" s="12"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="12"/>
+    </row>
+    <row r="25" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="B25" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="7"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="7" t="s">
+      <c r="C25" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D29" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="13" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="B33" s="13"/>
+      <c r="C33" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B32" s="11" t="s">
+    <row r="34" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B34" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D34" t="s">
         <v>36</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F34" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B36" s="7" t="s">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B40" s="7" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="7" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B44" s="13" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B46" s="13" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>